<commit_message>
SRIS-27: deleted descriptions of previousConfirmCode, highVolumeSite, mdardSoilVol from soil_relocation_receiving_sites.xlsx
</commit_message>
<xml_diff>
--- a/fields_description/soil_relocation_receiving_sites.xlsx
+++ b/fields_description/soil_relocation_receiving_sites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28014"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB_REPOS\nr-soils-relocation\fields_description\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{B2FD3C5A-3A58-4397-95F5-78BCF502BD09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02280F5C-3FF0-45C4-9EA5-571F58337BEF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C2ABF8-B69D-4943-B8D2-A59135465E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,10 +41,19 @@
     <author>Roy Jeong</author>
   </authors>
   <commentList>
-    <comment ref="A41" authorId="0" shapeId="0" xr:uid="{597AEDFB-653C-44DC-80F9-CF83BCA90FE0}">
+    <comment ref="A38" authorId="0" shapeId="0" xr:uid="{597AEDFB-653C-44DC-80F9-CF83BCA90FE0}">
       <text>
-        <t>Roy Jeong:
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Roy Jeong:
 Never rename fields. The field name is not incorrect, it is currently actually referenced as such in AGOL internally.</t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -52,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t>field</t>
   </si>
@@ -66,12 +75,6 @@
     <t>The confirmation ID is a number generated by the CHEFS form each time a soil relocation notification form is submitted. The number is used by submitters, First Nations, municipalities, members of the public and ministry staff to track individual submissions. The confirmation ID can also be used to request additional information from the soil relocation team. It is not editable.</t>
   </si>
   <si>
-    <t>previousConfirmCode</t>
-  </si>
-  <si>
-    <t>The field is used when the current soil relocation notification form is an update to a previous submission. If the submitter selects 'Yes' to indicate that the form is an update, they must enter the confirmation code of the previous submission in this field. For example, a valid entry might be '105A2Z1A'. This code corresponds to the confirmation ID generated by the CHEFS form for the earlier submission, enabling accurate tracking and reference.</t>
-  </si>
-  <si>
     <t>ownerCompany</t>
   </si>
   <si>
@@ -216,12 +219,6 @@
     <t>The field records the soil volume to be relocated (in cubic metres) for the wildlands reverted (WLR) soil quality. The data is a numerical value, and an example entry might be '13579'.</t>
   </si>
   <si>
-    <t>mdardSoilVol</t>
-  </si>
-  <si>
-    <t>The field records the soil volume to be relocated (in cubic metres) for soil quality without potential for Metals Leaching/Acid Rock Drainage (ML/ARD) as evaluated under Protocol 19. The data is a numerical value, and an example entry might be '13579'.</t>
-  </si>
-  <si>
     <t>totalSoilVolume</t>
   </si>
   <si>
@@ -244,12 +241,6 @@
   </si>
   <si>
     <t xml:space="preserve">The field displays how the relocated soil will be used at the receiving site, for example fill, cover, berms.  The format is text. </t>
-  </si>
-  <si>
-    <t>highVolumeSite</t>
-  </si>
-  <si>
-    <t>The field records whether the receiving site qualifies as a high volume site, defined as having more than 20,000 cubic metres of material deposited over its lifetime. The data is stored as 'Yes' or 'No', ensuring accurate classification of the site's volume status for tracking and regulatory purposes.</t>
   </si>
   <si>
     <t>soilDepositIsALR</t>
@@ -304,7 +295,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -691,14 +682,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
     <col min="2" max="2" width="121.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -706,7 +697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -714,7 +705,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -722,7 +713,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -730,7 +721,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -738,23 +729,23 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -762,7 +753,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -770,7 +761,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -778,7 +769,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -786,7 +777,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -794,7 +785,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -802,7 +793,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -810,7 +801,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -818,7 +809,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -826,7 +817,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -834,7 +825,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -842,7 +833,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -850,7 +841,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
@@ -858,7 +849,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -866,7 +857,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
@@ -874,15 +865,15 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>44</v>
       </c>
       <c r="B23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -890,7 +881,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -898,7 +889,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -906,7 +897,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -914,7 +905,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -922,7 +913,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>56</v>
       </c>
@@ -930,7 +921,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -938,7 +929,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -946,7 +937,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -954,7 +945,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>64</v>
       </c>
@@ -962,7 +953,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>66</v>
       </c>
@@ -970,7 +961,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -978,7 +969,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>70</v>
       </c>
@@ -986,7 +977,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>72</v>
       </c>
@@ -994,36 +985,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>74</v>
       </c>
       <c r="B38" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" t="s">
-        <v>76</v>
-      </c>
-      <c r="B39" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added notes into commercialSoilVol field
</commit_message>
<xml_diff>
--- a/fields_description/soil_relocation_receiving_sites.xlsx
+++ b/fields_description/soil_relocation_receiving_sites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB_REPOS\nr-soils-relocation\fields_description\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C2ABF8-B69D-4943-B8D2-A59135465E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17FDB640-7768-4203-8DE9-F167F594043D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="1500" windowWidth="31050" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,6 +41,30 @@
     <author>Roy Jeong</author>
   </authors>
   <commentList>
+    <comment ref="A20" authorId="0" shapeId="0" xr:uid="{C8C7EC40-E8C4-431B-A3E4-4E59D509E053}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Roy Jeong:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+When creating layer in AGOL, this field may be recognized only as a String type instead of a Double. In such cases, copy and paste from a locally created CSV file using a field name like ‘industrialSoilVol’ next to it, rename the field, delete the existing ‘commercialSoilVol’ field, save it, and then manually upload it to AGOL. This will allow the field to be recognized as a Double type.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="A38" authorId="0" shapeId="0" xr:uid="{597AEDFB-653C-44DC-80F9-CF83BCA90FE0}">
       <text>
         <r>
@@ -295,7 +319,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,6 +345,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>